<commit_message>
Changed bulk upload to use column based multi-select instead of row based fieldcapture#3676
</commit_message>
<xml_diff>
--- a/src/test/resources/bulk_import_example.xlsx
+++ b/src/test/resources/bulk_import_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/var03f/git/ecodata/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/god08d/projects/ecodata/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B769E5EA-E90F-E141-96BB-092F5B0496A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2837551D-2DD9-814C-A9D5-152432F9D6A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26560" xr2:uid="{2C3550E1-BCA6-BC4F-80D3-E9595D4DE580}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26200" xr2:uid="{2C3550E1-BCA6-BC4F-80D3-E9595D4DE580}"/>
   </bookViews>
   <sheets>
     <sheet name="form1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
   <si>
     <t>serial</t>
   </si>
@@ -59,9 +59,6 @@
     <t>bc</t>
   </si>
   <si>
-    <t>test bc 1</t>
-  </si>
-  <si>
     <t>test bc 2</t>
   </si>
   <si>
@@ -219,6 +216,9 @@
   </si>
   <si>
     <t>test bc 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test bc 1 </t>
   </si>
 </sst>
 </file>
@@ -590,21 +590,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2094674-6F1F-0348-B85A-E3F91D4F3835}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="25.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -615,37 +615,46 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" t="s">
-        <v>20</v>
-      </c>
       <c r="H1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="J1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N1" t="s">
         <v>46</v>
       </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>47</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>48</v>
       </c>
-      <c r="M1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -656,233 +665,242 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="I2" t="s">
-        <v>45</v>
-      </c>
-      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
       <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" t="s">
         <v>26</v>
       </c>
-      <c r="I3" t="s">
+      <c r="P3" t="s">
         <v>50</v>
       </c>
-      <c r="J3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
-      </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="I5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" t="s">
         <v>53</v>
       </c>
-      <c r="J5" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L5" t="s">
-        <v>31</v>
-      </c>
-      <c r="M5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" t="s">
-        <v>40</v>
-      </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" t="s">
         <v>55</v>
       </c>
-      <c r="J6" t="s">
-        <v>40</v>
-      </c>
-      <c r="K6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L6" t="s">
-        <v>38</v>
-      </c>
-      <c r="M6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2</v>
       </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" t="s">
-        <v>37</v>
-      </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+      <c r="M7" t="s">
+        <v>40</v>
+      </c>
+      <c r="N7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O7" t="s">
+        <v>38</v>
+      </c>
+      <c r="P7" t="s">
         <v>57</v>
       </c>
-      <c r="J7" t="s">
-        <v>41</v>
-      </c>
-      <c r="K7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3</v>
       </c>
       <c r="B8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
         <v>59</v>
       </c>
-      <c r="C8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>

</xml_diff>